<commit_message>
fix(esg-profile): complete anonymization scrub, externalize denylist, genericize skill, align fund fixture
</commit_message>
<xml_diff>
--- a/skills/esg-profile/demo/static/extract.xlsx
+++ b/skills/esg-profile/demo/static/extract.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Net Zero policy not yet formalized (in progress); green lease language absent — multi-year regression; climate adaptation plan absent — multi-year regression; embodied carbon at 0% of assets — regression; employee engagement program informal only — regression; energy data coverage at Fund VII level 19% vs MIR 27%; physical risk: Moderate (Wind, Heat, Drought — Spain)</t>
+          <t>Net Zero policy not yet formalized (in progress); green lease language absent — multi-year regression; climate adaptation plan absent — multi-year regression; embodied carbon at 0% of assets — regression; employee engagement program informal only — regression; energy data coverage at Fund VII level 19% vs MIR 27%; physical risk: Moderate (Wind, Heat, Drought — Southern Europe)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC upgrade requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs; UNGC (10th and 3rd principles); OECD BEPS</t>
+          <t>national energy-efficiency regulations; EPC upgrade requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs; UNGC (10th and 3rd principles); OECD BEPS</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Net Zero policy not yet formalized (in progress); green lease language absent — multi-year regression; climate adaptation plan absent — multi-year regression; embodied carbon at 0% of assets — regression; employee engagement program informal only — regression; energy data coverage at Fund VII level 19% vs MIR 27%; physical risk: Moderate (Wind, Heat, Drought — Spain)</t>
+          <t>Net Zero policy not yet formalized (in progress); green lease language absent — multi-year regression; climate adaptation plan absent — multi-year regression; embodied carbon at 0% of assets — regression; employee engagement program informal only — regression; energy data coverage at Fund VII level 19% vs MIR 27%; physical risk: Moderate (Wind, Heat, Drought — Southern Europe)</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC upgrade requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs; UNGC (10th and 3rd principles); OECD BEPS</t>
+          <t>national energy-efficiency regulations; EPC upgrade requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs; UNGC (10th and 3rd principles); OECD BEPS</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Project EREB EPC upgrade program ($30M budget, 20 assets E→C by 2025/2026); CRREM portfolio-wide stranding analysis; BREEAM-Use certifications via Alma; gas-to-electric switching; Hoop carpooling app pilot; EV charger rollout via tenant app</t>
+          <t>Project EREB EPC upgrade program ($30M budget, 20 assets E→C by 2025/2026); CRREM portfolio-wide stranding analysis; BREEAM-Use certifications via a third-party consultant; gas-to-electric switching; Hoop carpooling app pilot; EV charger rollout via tenant app</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
+          <t>national energy-efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Project EREB EPC upgrade program ($30M budget, 20 assets E→C by 2025/2026); CRREM portfolio-wide stranding analysis; BREEAM-Use certifications via Alma; gas-to-electric switching; Hoop carpooling app pilot; EV charger rollout via tenant app</t>
+          <t>Project EREB EPC upgrade program ($30M budget, 20 assets E→C by 2025/2026); CRREM portfolio-wide stranding analysis; BREEAM-Use certifications via a third-party consultant; gas-to-electric switching; Hoop carpooling app pilot; EV charger rollout via tenant app</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
+          <t>national energy-efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
+          <t>national energy-efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Spanish energy efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
+          <t>national energy-efficiency regulations; EPC requirements; GRESB; TCFD; GRI; UN PRI; UN SDGs</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">

</xml_diff>